<commit_message>
Added the printer to the BOM.
</commit_message>
<xml_diff>
--- a/system_development/Pintail/V1.1.1/BOM-Pintail_v0.1.1.xlsx
+++ b/system_development/Pintail/V1.1.1/BOM-Pintail_v0.1.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/austindowney/Documents/GitHub/FUSE-Head/system_development/Pintail/V1.1.1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jacob Parker\Documents\GitHub\FUSE-Head\system_development\Pintail\V1.1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DA60863-2180-9E4D-AC80-DD5387B7A6EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD9676F9-CE85-46D6-BA3A-4CF9541C5451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
+    <workbookView xWindow="14220" yWindow="-150" windowWidth="14835" windowHeight="15885" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="bill_of_materials" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4294966976" uniqueCount="33">
   <si>
     <t>Individual Cost</t>
   </si>
@@ -120,6 +120,21 @@
   </si>
   <si>
     <t>Primary</t>
+  </si>
+  <si>
+    <t>Creality/eBay</t>
+  </si>
+  <si>
+    <t>Ender-3 V3 se</t>
+  </si>
+  <si>
+    <t>https://ebay.io/m/1bKKzi</t>
+  </si>
+  <si>
+    <t>https://store.creality.com/products/ender-3-v3-se-3d-printer?spm=..product_accf228c-979f-450e-90b4-4d88e008979f.0.1</t>
+  </si>
+  <si>
+    <t>3D printer</t>
   </si>
 </sst>
 </file>
@@ -609,24 +624,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
   <dimension ref="A1:N22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="27.33203125" customWidth="1"/>
-    <col min="3" max="3" width="37.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="27.28515625" customWidth="1"/>
+    <col min="3" max="3" width="37.85546875" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
     <col min="9" max="9" width="79" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="45.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="83.5" customWidth="1"/>
-    <col min="12" max="12" width="62.5" customWidth="1"/>
-    <col min="13" max="13" width="55.83203125" customWidth="1"/>
+    <col min="10" max="10" width="45.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="83.42578125" customWidth="1"/>
+    <col min="12" max="12" width="62.42578125" customWidth="1"/>
+    <col min="13" max="13" width="55.85546875" customWidth="1"/>
     <col min="14" max="14" width="51" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>10</v>
       </c>
@@ -670,7 +685,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>24</v>
       </c>
@@ -699,7 +714,7 @@
       </c>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
         <v>15</v>
       </c>
@@ -728,7 +743,7 @@
       </c>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -759,20 +774,39 @@
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
     </row>
-    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="17"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
+    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="19">
+        <v>1</v>
+      </c>
+      <c r="F5" s="9">
+        <v>75</v>
+      </c>
+      <c r="G5" s="9">
+        <v>75</v>
+      </c>
       <c r="H5" s="5"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="4"/>
+      <c r="I5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>30</v>
+      </c>
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
     </row>
-    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="17"/>
       <c r="C6" s="2"/>
       <c r="D6" s="20"/>
@@ -780,9 +814,8 @@
       <c r="F6" s="9"/>
       <c r="G6" s="9"/>
       <c r="H6" s="5"/>
-      <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10"/>
       <c r="B7" s="17"/>
       <c r="C7" s="2"/>
@@ -794,7 +827,7 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" s="17"/>
       <c r="C8" s="2"/>
@@ -806,7 +839,7 @@
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
     </row>
-    <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
       <c r="C9" s="2"/>
@@ -818,7 +851,7 @@
       <c r="I9" s="1"/>
       <c r="J9" s="4"/>
     </row>
-    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
       <c r="B10" s="17"/>
       <c r="C10" s="2"/>
@@ -830,7 +863,7 @@
       <c r="I10" s="1"/>
       <c r="J10" s="4"/>
     </row>
-    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="B11" s="17"/>
       <c r="C11" s="4"/>
@@ -842,7 +875,7 @@
       <c r="I11" s="1"/>
       <c r="J11" s="4"/>
     </row>
-    <row r="12" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10"/>
       <c r="B12" s="17"/>
       <c r="C12" s="2"/>
@@ -854,7 +887,7 @@
       <c r="I12" s="1"/>
       <c r="J12" s="4"/>
     </row>
-    <row r="13" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10"/>
       <c r="B13" s="17"/>
       <c r="C13" s="2"/>
@@ -866,7 +899,7 @@
       <c r="I13" s="1"/>
       <c r="J13" s="4"/>
     </row>
-    <row r="14" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10"/>
       <c r="B14" s="17"/>
       <c r="C14" s="2"/>
@@ -878,7 +911,7 @@
       <c r="I14" s="1"/>
       <c r="J14" s="4"/>
     </row>
-    <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10"/>
       <c r="B15" s="17"/>
       <c r="C15" s="2"/>
@@ -889,7 +922,7 @@
       <c r="H15" s="5"/>
       <c r="I15" s="1"/>
     </row>
-    <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
       <c r="C16" s="2"/>
@@ -901,7 +934,7 @@
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
     </row>
-    <row r="17" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="17"/>
       <c r="C17" s="2"/>
@@ -913,7 +946,7 @@
       <c r="I17" s="3"/>
       <c r="J17" s="4"/>
     </row>
-    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11"/>
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
@@ -926,7 +959,7 @@
       <c r="J18" s="11"/>
       <c r="K18" s="11"/>
     </row>
-    <row r="19" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11"/>
       <c r="B19" s="11"/>
       <c r="C19" s="11"/>
@@ -938,7 +971,7 @@
       <c r="J19" s="11"/>
       <c r="K19" s="11"/>
     </row>
-    <row r="20" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -949,17 +982,17 @@
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F21" s="8"/>
       <c r="G21" s="8"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F22" s="7" t="s">
         <v>7</v>
       </c>
       <c r="G22" s="5">
         <f>SUM(G2:G21)</f>
-        <v>92.51</v>
+        <v>167.51</v>
       </c>
     </row>
   </sheetData>
@@ -968,8 +1001,9 @@
     <hyperlink ref="I2" r:id="rId1" xr:uid="{47569AE6-6AA0-4875-B93F-ACB3A5943EC4}"/>
     <hyperlink ref="I3" r:id="rId2" xr:uid="{D098FC55-60BA-44A1-88B5-F7A95F7F2234}"/>
     <hyperlink ref="I4" r:id="rId3" xr:uid="{E4B64C1A-2E26-4C6F-9252-C15670A96A6B}"/>
+    <hyperlink ref="I5" r:id="rId4" tooltip="Original URL: https://store.creality.com/products/ender-3-v3-se-3d-printer?spm=..product_accf228c-979f-450e-90b4-4d88e008979f.0.1. Click or tap if you trust this link." display="https://nam02.safelinks.protection.outlook.com/?url=https%3A%2F%2Fstore.creality.com%2Fproducts%2Fender-3-v3-se-3d-printer%3Fspm%3D..product_accf228c-979f-450e-90b4-4d88e008979f.0.1&amp;data=05%7C02%7CJHPARKER%40email.sc.edu%7Ca352611c2134487fcf1808df150dcc02%7C4b2a4b19d135420e8bb2b1cd238998cc%7C0%7C0%7C639252821129488256%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=VJaeAAT8rnG%2FPhk3%2Bme9G0Ml1MFBbcEWWrzPLMmHcYQ%3D&amp;reserved=0" xr:uid="{27A3E46D-50E1-4DC7-B0D5-E25881E90590}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>